<commit_message>
Fix portable UAV doc export and Diff-planner path
</commit_message>
<xml_diff>
--- a/docs/非凸α-素材缺口表.xlsx
+++ b/docs/非凸α-素材缺口表.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="素材缺口表" sheetId="1" r:id="Rac9b787a191b486e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怎么用" sheetId="1" r:id="R6bed98d242284f83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="缺口明细" sheetId="2" r:id="R785ec049c3af469b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,28 +14,156 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="1">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color theme="0"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="444444"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="13"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color theme="0"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="2">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor theme="4" tint="0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor theme="5" tint="0.35"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor theme="4"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="9">
     <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="D9D9D9"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="D9D9D9"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="D9D9D9"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="D9D9D9"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="D9D9D9"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="D9D9D9"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="D9D9D9"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="D9D9D9"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="D9D9D9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="D9D9D9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="D9D9D9"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="D9D9D9"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -190,188 +319,309 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23.93000030517578" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="43.560001373291016" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" t="str">
-        <x:v>state_group</x:v>
-      </x:c>
-      <x:c r="B1" t="str">
-        <x:v>required_shot</x:v>
-      </x:c>
-      <x:c r="C1" t="str">
-        <x:v>currently_available</x:v>
-      </x:c>
-      <x:c r="D1" t="str">
-        <x:v>evidence_source</x:v>
-      </x:c>
-      <x:c r="E1" t="str">
-        <x:v>gap_reason</x:v>
-      </x:c>
-      <x:c r="F1" t="str">
-        <x:v>collection_instruction</x:v>
-      </x:c>
-      <x:c r="G1" t="str">
-        <x:v>priority</x:v>
-      </x:c>
+      <x:c r="A1" s="2" t="str">
+        <x:v>素材缺口表怎么用</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
+      <x:c r="A2" s="4" t="str">
+        <x:v>这一份不是开发接口表，而是给后续补截图、补培训材料的人用。P0 先补，P1 次之。</x:v>
+      </x:c>
+      <x:c r="B2" s="4"/>
+      <x:c r="C2" s="4"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="6" t="str">
+        <x:v>阅读方式</x:v>
+      </x:c>
+      <x:c r="B4" s="6"/>
+      <x:c r="C4" s="6"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="9" t="str">
+        <x:v>你想做什么</x:v>
+      </x:c>
+      <x:c r="B5" s="9" t="str">
+        <x:v>看哪里</x:v>
+      </x:c>
+      <x:c r="C5" s="9" t="str">
+        <x:v>说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="10" t="str">
+        <x:v>确定先补哪些截图</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>优先级列</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
+        <x:v>P0 是当前最影响日常使用的缺口。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="13" t="str">
+        <x:v>知道每张图为什么缺</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="str">
+        <x:v>缺口明细</x:v>
+      </x:c>
+      <x:c r="C7" s="14" t="str">
+        <x:v>这里把缺口原因和补采指令写清楚了。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="15" t="str">
+        <x:v>准备拍摄任务</x:v>
+      </x:c>
+      <x:c r="B8" s="16" t="str">
+        <x:v>缺口明细</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>直接按 collection_instruction 执行。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23.93000030517578" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11.65999984741211" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>缺口明细</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="4" t="str">
+        <x:v>这些缺口对应的是仍需补拍或补标注的日常使用素材。</x:v>
+      </x:c>
+      <x:c r="B2" s="4"/>
+      <x:c r="C2" s="4"/>
+      <x:c r="D2" s="4"/>
+      <x:c r="E2" s="4"/>
+      <x:c r="F2" s="4"/>
+      <x:c r="G2" s="4"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="6" t="str">
+        <x:v>素材缺口</x:v>
+      </x:c>
+      <x:c r="B4" s="6"/>
+      <x:c r="C4" s="6"/>
+      <x:c r="D4" s="6"/>
+      <x:c r="E4" s="6"/>
+      <x:c r="F4" s="6"/>
+      <x:c r="G4" s="6"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="9" t="str">
+        <x:v>状态场景</x:v>
+      </x:c>
+      <x:c r="B5" s="9" t="str">
+        <x:v>需要补什么</x:v>
+      </x:c>
+      <x:c r="C5" s="9" t="str">
+        <x:v>当前情况</x:v>
+      </x:c>
+      <x:c r="D5" s="9" t="str">
+        <x:v>证据来源</x:v>
+      </x:c>
+      <x:c r="E5" s="9" t="str">
+        <x:v>为什么缺</x:v>
+      </x:c>
+      <x:c r="F5" s="9" t="str">
+        <x:v>补采指令</x:v>
+      </x:c>
+      <x:c r="G5" s="9" t="str">
+        <x:v>优先级</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="10" t="str">
         <x:v>起飞前</x:v>
       </x:c>
-      <x:c r="B2" t="str">
+      <x:c r="B6" s="11" t="str">
         <x:v>遥控器全景+5/6/7/8 通档位</x:v>
       </x:c>
-      <x:c r="C2" t="str">
+      <x:c r="C6" s="11" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="D2" t="str">
+      <x:c r="D6" s="11" t="str">
         <x:v>本地知识库与 PDF</x:v>
       </x:c>
-      <x:c r="E2" t="str">
+      <x:c r="E6" s="11" t="str">
         <x:v>现有资料只有文字说明且未集中标注档位</x:v>
       </x:c>
-      <x:c r="F2" t="str">
+      <x:c r="F6" s="11" t="str">
         <x:v>补拍遥控器正视图并在图上标明 5/6/7/8 通位置和含义</x:v>
       </x:c>
-      <x:c r="G2" t="str">
+      <x:c r="G6" s="12" t="str">
         <x:v>P0</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" t="str">
+    <x:row r="7">
+      <x:c r="A7" s="13" t="str">
         <x:v>起飞前</x:v>
       </x:c>
-      <x:c r="B3" t="str">
+      <x:c r="B7" s="3" t="str">
         <x:v>终端中 /mavros/state + /mavros/battery + /mavros/rc/in 三联观测</x:v>
       </x:c>
-      <x:c r="C3" t="str">
+      <x:c r="C7" s="3" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="D3" t="str">
+      <x:c r="D7" s="3" t="str">
         <x:v>本地知识库 05/06 章</x:v>
       </x:c>
-      <x:c r="E3" t="str">
+      <x:c r="E7" s="3" t="str">
         <x:v>只有命令没有统一截图</x:v>
       </x:c>
-      <x:c r="F3" t="str">
+      <x:c r="F7" s="3" t="str">
         <x:v>补拍三个终端或 tmux 分屏画面并保留时间戳</x:v>
       </x:c>
-      <x:c r="G3" t="str">
+      <x:c r="G7" s="14" t="str">
         <x:v>P0</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
+    <x:row r="8">
+      <x:c r="A8" s="13" t="str">
         <x:v>手动悬停与接管</x:v>
       </x:c>
-      <x:c r="B4" t="str">
+      <x:c r="B8" s="3" t="str">
         <x:v>6 通上拨后的安全兜底状态</x:v>
       </x:c>
-      <x:c r="C4" t="str">
+      <x:c r="C8" s="3" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="D4" t="str">
+      <x:c r="D8" s="3" t="str">
         <x:v>本地知识库 01 章</x:v>
       </x:c>
-      <x:c r="E4" t="str">
+      <x:c r="E8" s="3" t="str">
         <x:v>缺少接管前后对照图</x:v>
       </x:c>
-      <x:c r="F4" t="str">
+      <x:c r="F8" s="3" t="str">
         <x:v>补拍悬停状态下的 RC 档位和 rviz/终端画面</x:v>
       </x:c>
-      <x:c r="G4" t="str">
+      <x:c r="G8" s="14" t="str">
         <x:v>P0</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str">
+    <x:row r="9">
+      <x:c r="A9" s="13" t="str">
         <x:v>自主执行</x:v>
       </x:c>
-      <x:c r="B5" t="str">
+      <x:c r="B9" s="3" t="str">
         <x:v>LIO 任务执行中的轨迹和点云画面</x:v>
       </x:c>
-      <x:c r="C5" t="str">
+      <x:c r="C9" s="3" t="str">
         <x:v>partial</x:v>
       </x:c>
-      <x:c r="D5" t="str">
+      <x:c r="D9" s="3" t="str">
         <x:v>Diff-planner images + 本地知识库</x:v>
       </x:c>
-      <x:c r="E5" t="str">
+      <x:c r="E9" s="3" t="str">
         <x:v>现有 gif 更偏算法展示没有开发判断点标注</x:v>
       </x:c>
-      <x:c r="F5" t="str">
+      <x:c r="F9" s="3" t="str">
         <x:v>补加标注或重截更清晰的实机 rviz 画面</x:v>
       </x:c>
-      <x:c r="G5" t="str">
+      <x:c r="G9" s="14" t="str">
         <x:v>P1</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="13" t="str">
         <x:v>自主执行</x:v>
       </x:c>
-      <x:c r="B6" t="str">
+      <x:c r="B10" s="3" t="str">
         <x:v>VIO 任务执行中的相机/VINS/轨迹联合画面</x:v>
       </x:c>
-      <x:c r="C6" t="str">
+      <x:c r="C10" s="3" t="str">
         <x:v>partial</x:v>
       </x:c>
-      <x:c r="D6" t="str">
+      <x:c r="D10" s="3" t="str">
         <x:v>本地知识库 04/05 章</x:v>
       </x:c>
-      <x:c r="E6" t="str">
+      <x:c r="E10" s="3" t="str">
         <x:v>只有文字和零散图没有联合视图</x:v>
       </x:c>
-      <x:c r="F6" t="str">
+      <x:c r="F10" s="3" t="str">
         <x:v>补拍相机图像 + odom + rviz 联合画面</x:v>
       </x:c>
-      <x:c r="G6" t="str">
+      <x:c r="G10" s="14" t="str">
         <x:v>P1</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
+    <x:row r="11">
+      <x:c r="A11" s="13" t="str">
         <x:v>返航与降落</x:v>
       </x:c>
-      <x:c r="B7" t="str">
+      <x:c r="B11" s="3" t="str">
         <x:v>返航触发前后对照</x:v>
       </x:c>
-      <x:c r="C7" t="str">
+      <x:c r="C11" s="3" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="D7" t="str">
+      <x:c r="D11" s="3" t="str">
         <x:v>脚本与 RC 映射源码</x:v>
       </x:c>
-      <x:c r="E7" t="str">
+      <x:c r="E11" s="3" t="str">
         <x:v>缺少返航触发前后状态画面</x:v>
       </x:c>
-      <x:c r="F7" t="str">
+      <x:c r="F11" s="3" t="str">
         <x:v>补拍返航触发瞬间和返航中状态</x:v>
       </x:c>
-      <x:c r="G7" t="str">
+      <x:c r="G11" s="14" t="str">
         <x:v>P1</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
+    <x:row r="12">
+      <x:c r="A12" s="15" t="str">
         <x:v>返航与降落</x:v>
       </x:c>
-      <x:c r="B8" t="str">
+      <x:c r="B12" s="16" t="str">
         <x:v>自动降落完成后落地判定画面</x:v>
       </x:c>
-      <x:c r="C8" t="str">
+      <x:c r="C12" s="16" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="D8" t="str">
+      <x:c r="D12" s="16" t="str">
         <x:v>脚本与状态 topic</x:v>
       </x:c>
-      <x:c r="E8" t="str">
+      <x:c r="E12" s="16" t="str">
         <x:v>缺少动作结束示例</x:v>
       </x:c>
-      <x:c r="F8" t="str">
+      <x:c r="F12" s="16" t="str">
         <x:v>补拍落地后状态与终端提示并标注结束判据</x:v>
       </x:c>
-      <x:c r="G8" t="str">
+      <x:c r="G12" s="17" t="str">
         <x:v>P1</x:v>
       </x:c>
     </x:row>

</xml_diff>